<commit_message>
so many images added
</commit_message>
<xml_diff>
--- a/Documents/Product Catalog/Steel Almirah.xlsx
+++ b/Documents/Product Catalog/Steel Almirah.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Talukder Furniture\Documents\Product Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6FBE23-31D2-4032-B0E0-BD9D4DD87F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Steel Almirah" sheetId="5" r:id="rId1"/>
@@ -17,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Steel Almirah'!$A$1:$Q$20</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -289,7 +303,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="9">
     <font>
       <sz val="10"/>
@@ -588,22 +602,34 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -617,18 +643,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,7 +841,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="16"/>
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
@@ -836,7 +850,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="11"/>
       <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
       <tableStyleElement type="firstRowStripe" dxfId="7"/>
@@ -875,7 +889,7 @@
         <xdr:cNvPr id="2" name="image1.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000048010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000048010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -925,7 +939,7 @@
         <xdr:cNvPr id="65" name="image313.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000049010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000049010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -975,7 +989,7 @@
         <xdr:cNvPr id="66" name="image314.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00004A010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004A010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1025,7 +1039,7 @@
         <xdr:cNvPr id="67" name="image315.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00004B010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004B010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1075,7 +1089,7 @@
         <xdr:cNvPr id="68" name="image316.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00004C010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004C010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1125,7 +1139,7 @@
         <xdr:cNvPr id="69" name="image317.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00004D010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004D010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1175,7 +1189,7 @@
         <xdr:cNvPr id="70" name="image318.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00004E010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004E010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1225,7 +1239,7 @@
         <xdr:cNvPr id="71" name="image319.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00004F010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004F010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1275,7 +1289,7 @@
         <xdr:cNvPr id="72" name="image320.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000050010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000050010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1325,7 +1339,7 @@
         <xdr:cNvPr id="73" name="Group 355">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000051010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000051010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1333,7 +1347,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4498081" y="10151272"/>
+          <a:off x="4487195" y="10175765"/>
           <a:ext cx="499142" cy="887522"/>
           <a:chOff x="0" y="0"/>
           <a:chExt cx="331470" cy="635000"/>
@@ -1344,7 +1358,7 @@
           <xdr:cNvPr id="74" name="image321.png">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000052010000}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000052010000}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1379,7 +1393,7 @@
           <xdr:cNvPr id="75" name="image322.jpeg">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000053010000}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000053010000}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1430,7 +1444,7 @@
         <xdr:cNvPr id="76" name="image323.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000054010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000054010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1480,7 +1494,7 @@
         <xdr:cNvPr id="77" name="image324.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000055010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000055010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1530,7 +1544,7 @@
         <xdr:cNvPr id="78" name="image325.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000056010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000056010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1580,7 +1594,7 @@
         <xdr:cNvPr id="79" name="image327.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000057010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000057010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1630,7 +1644,7 @@
         <xdr:cNvPr id="80" name="image328.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000058010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000058010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1680,7 +1694,7 @@
         <xdr:cNvPr id="81" name="image325.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00005F010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00005F010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1730,7 +1744,7 @@
         <xdr:cNvPr id="82" name="image325.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000060010000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000060010000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2014,7 +2028,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AT130"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
@@ -2039,49 +2053,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
     </row>
     <row r="2" spans="1:46" ht="39.950000000000003" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="29"/>
     </row>
     <row r="3" spans="1:46" ht="50.1" customHeight="1">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="30" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="24" t="s">
@@ -2090,21 +2104,21 @@
       <c r="C3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="32" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="31"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="27"/>
       <c r="I3" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="28" t="s">
+      <c r="J3" s="32" t="s">
         <v>9</v>
       </c>
       <c r="K3" s="24" t="s">
@@ -2154,11 +2168,11 @@
       <c r="AT3" s="4"/>
     </row>
     <row r="4" spans="1:46" ht="33.200000000000003" customHeight="1">
-      <c r="A4" s="27"/>
+      <c r="A4" s="31"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="F4" s="21" t="s">
         <v>13</v>
       </c>
@@ -2169,7 +2183,7 @@
         <v>61</v>
       </c>
       <c r="I4" s="24"/>
-      <c r="J4" s="29"/>
+      <c r="J4" s="33"/>
       <c r="K4" s="5" t="s">
         <v>15</v>
       </c>
@@ -2249,7 +2263,7 @@
         <v>28500</v>
       </c>
       <c r="M5" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N5" s="17" t="s">
         <v>42</v>
@@ -2301,7 +2315,7 @@
         <v>28500</v>
       </c>
       <c r="M6" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N6" s="17" t="s">
         <v>46</v>
@@ -2353,7 +2367,7 @@
         <v>28500</v>
       </c>
       <c r="M7" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N7" s="17" t="s">
         <v>47</v>
@@ -2405,7 +2419,7 @@
         <v>28500</v>
       </c>
       <c r="M8" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N8" s="17" t="s">
         <v>48</v>
@@ -2457,7 +2471,7 @@
         <v>28500</v>
       </c>
       <c r="M9" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N9" s="17" t="s">
         <v>49</v>
@@ -2509,7 +2523,7 @@
         <v>28500</v>
       </c>
       <c r="M10" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N10" s="17" t="s">
         <v>50</v>
@@ -2561,7 +2575,7 @@
         <v>28500</v>
       </c>
       <c r="M11" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N11" s="17" t="s">
         <v>51</v>
@@ -2613,7 +2627,7 @@
         <v>28500</v>
       </c>
       <c r="M12" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N12" s="17" t="s">
         <v>52</v>
@@ -2665,7 +2679,7 @@
         <v>28500</v>
       </c>
       <c r="M13" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N13" s="17" t="s">
         <v>53</v>
@@ -2717,7 +2731,7 @@
         <v>28500</v>
       </c>
       <c r="M14" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N14" s="17" t="s">
         <v>54</v>
@@ -2769,7 +2783,7 @@
         <v>28500</v>
       </c>
       <c r="M15" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N15" s="17" t="s">
         <v>55</v>
@@ -2821,7 +2835,7 @@
         <v>28500</v>
       </c>
       <c r="M16" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N16" s="17" t="s">
         <v>56</v>
@@ -2873,7 +2887,7 @@
         <v>28500</v>
       </c>
       <c r="M17" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N17" s="17" t="s">
         <v>57</v>
@@ -2925,7 +2939,7 @@
         <v>28500</v>
       </c>
       <c r="M18" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N18" s="17" t="s">
         <v>58</v>
@@ -2977,7 +2991,7 @@
         <v>28500</v>
       </c>
       <c r="M19" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N19" s="17" t="s">
         <v>59</v>
@@ -3029,7 +3043,7 @@
         <v>28500</v>
       </c>
       <c r="M20" s="10">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="N20" s="17" t="s">
         <v>60</v>
@@ -3045,24 +3059,24 @@
       </c>
     </row>
     <row r="21" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A21" s="32"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="33"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
-      <c r="N21" s="33"/>
-      <c r="O21" s="33"/>
-      <c r="P21" s="33"/>
-      <c r="Q21" s="33"/>
-      <c r="R21" s="33"/>
+      <c r="A21" s="22"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
+      <c r="N21" s="23"/>
+      <c r="O21" s="23"/>
+      <c r="P21" s="23"/>
+      <c r="Q21" s="23"/>
+      <c r="R21" s="23"/>
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
       <c r="U21" s="4"/>
@@ -3093,24 +3107,24 @@
       <c r="AT21" s="4"/>
     </row>
     <row r="22" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A22" s="32"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="33"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="33"/>
-      <c r="O22" s="33"/>
-      <c r="P22" s="33"/>
-      <c r="Q22" s="33"/>
-      <c r="R22" s="33"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="23"/>
+      <c r="O22" s="23"/>
+      <c r="P22" s="23"/>
+      <c r="Q22" s="23"/>
+      <c r="R22" s="23"/>
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
       <c r="U22" s="4"/>
@@ -3141,24 +3155,24 @@
       <c r="AT22" s="4"/>
     </row>
     <row r="23" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A23" s="32"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="33"/>
-      <c r="J23" s="33"/>
-      <c r="K23" s="33"/>
-      <c r="L23" s="33"/>
-      <c r="M23" s="33"/>
-      <c r="N23" s="33"/>
-      <c r="O23" s="33"/>
-      <c r="P23" s="33"/>
-      <c r="Q23" s="33"/>
-      <c r="R23" s="33"/>
+      <c r="A23" s="22"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="23"/>
+      <c r="O23" s="23"/>
+      <c r="P23" s="23"/>
+      <c r="Q23" s="23"/>
+      <c r="R23" s="23"/>
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
@@ -3189,24 +3203,24 @@
       <c r="AT23" s="4"/>
     </row>
     <row r="24" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A24" s="32"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33"/>
-      <c r="Q24" s="33"/>
-      <c r="R24" s="33"/>
+      <c r="A24" s="22"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
+      <c r="N24" s="23"/>
+      <c r="O24" s="23"/>
+      <c r="P24" s="23"/>
+      <c r="Q24" s="23"/>
+      <c r="R24" s="23"/>
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
       <c r="U24" s="4"/>
@@ -3237,24 +3251,24 @@
       <c r="AT24" s="4"/>
     </row>
     <row r="25" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A25" s="32"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
-      <c r="N25" s="33"/>
-      <c r="O25" s="33"/>
-      <c r="P25" s="33"/>
-      <c r="Q25" s="33"/>
-      <c r="R25" s="33"/>
+      <c r="A25" s="22"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="23"/>
+      <c r="O25" s="23"/>
+      <c r="P25" s="23"/>
+      <c r="Q25" s="23"/>
+      <c r="R25" s="23"/>
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
       <c r="U25" s="4"/>
@@ -3285,24 +3299,24 @@
       <c r="AT25" s="4"/>
     </row>
     <row r="26" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A26" s="32"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="33"/>
-      <c r="P26" s="33"/>
-      <c r="Q26" s="33"/>
-      <c r="R26" s="33"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="23"/>
+      <c r="R26" s="23"/>
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
       <c r="U26" s="4"/>
@@ -3333,24 +3347,24 @@
       <c r="AT26" s="4"/>
     </row>
     <row r="27" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A27" s="32"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="33"/>
-      <c r="P27" s="33"/>
-      <c r="Q27" s="33"/>
-      <c r="R27" s="33"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="23"/>
+      <c r="O27" s="23"/>
+      <c r="P27" s="23"/>
+      <c r="Q27" s="23"/>
+      <c r="R27" s="23"/>
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
       <c r="U27" s="4"/>
@@ -3381,24 +3395,24 @@
       <c r="AT27" s="4"/>
     </row>
     <row r="28" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A28" s="32"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="33"/>
-      <c r="O28" s="33"/>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="33"/>
-      <c r="R28" s="33"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="23"/>
+      <c r="Q28" s="23"/>
+      <c r="R28" s="23"/>
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
       <c r="U28" s="4"/>
@@ -3429,24 +3443,24 @@
       <c r="AT28" s="4"/>
     </row>
     <row r="29" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A29" s="32"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="33"/>
-      <c r="J29" s="33"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
-      <c r="M29" s="33"/>
-      <c r="N29" s="33"/>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33"/>
-      <c r="Q29" s="33"/>
-      <c r="R29" s="33"/>
+      <c r="A29" s="22"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
+      <c r="K29" s="23"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="23"/>
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
+      <c r="P29" s="23"/>
+      <c r="Q29" s="23"/>
+      <c r="R29" s="23"/>
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
       <c r="U29" s="4"/>
@@ -3477,24 +3491,24 @@
       <c r="AT29" s="4"/>
     </row>
     <row r="30" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A30" s="32"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="33"/>
-      <c r="D30" s="33"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="33"/>
-      <c r="K30" s="33"/>
-      <c r="L30" s="33"/>
-      <c r="M30" s="33"/>
-      <c r="N30" s="33"/>
-      <c r="O30" s="33"/>
-      <c r="P30" s="33"/>
-      <c r="Q30" s="33"/>
-      <c r="R30" s="33"/>
+      <c r="A30" s="22"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="23"/>
+      <c r="N30" s="23"/>
+      <c r="O30" s="23"/>
+      <c r="P30" s="23"/>
+      <c r="Q30" s="23"/>
+      <c r="R30" s="23"/>
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
       <c r="U30" s="4"/>
@@ -3525,24 +3539,24 @@
       <c r="AT30" s="4"/>
     </row>
     <row r="31" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A31" s="32"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="33"/>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
-      <c r="O31" s="33"/>
-      <c r="P31" s="33"/>
-      <c r="Q31" s="33"/>
-      <c r="R31" s="33"/>
+      <c r="A31" s="22"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+      <c r="P31" s="23"/>
+      <c r="Q31" s="23"/>
+      <c r="R31" s="23"/>
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
       <c r="U31" s="4"/>
@@ -3573,24 +3587,24 @@
       <c r="AT31" s="4"/>
     </row>
     <row r="32" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A32" s="32"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="33"/>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="33"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
-      <c r="I32" s="33"/>
-      <c r="J32" s="33"/>
-      <c r="K32" s="33"/>
-      <c r="L32" s="33"/>
-      <c r="M32" s="33"/>
-      <c r="N32" s="33"/>
-      <c r="O32" s="33"/>
-      <c r="P32" s="33"/>
-      <c r="Q32" s="33"/>
-      <c r="R32" s="33"/>
+      <c r="A32" s="22"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
+      <c r="O32" s="23"/>
+      <c r="P32" s="23"/>
+      <c r="Q32" s="23"/>
+      <c r="R32" s="23"/>
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
       <c r="U32" s="4"/>
@@ -3621,24 +3635,24 @@
       <c r="AT32" s="4"/>
     </row>
     <row r="33" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A33" s="32"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="33"/>
-      <c r="J33" s="33"/>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
-      <c r="N33" s="33"/>
-      <c r="O33" s="33"/>
-      <c r="P33" s="33"/>
-      <c r="Q33" s="33"/>
-      <c r="R33" s="33"/>
+      <c r="A33" s="22"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="23"/>
+      <c r="N33" s="23"/>
+      <c r="O33" s="23"/>
+      <c r="P33" s="23"/>
+      <c r="Q33" s="23"/>
+      <c r="R33" s="23"/>
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
       <c r="U33" s="4"/>
@@ -3669,24 +3683,24 @@
       <c r="AT33" s="4"/>
     </row>
     <row r="34" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A34" s="32"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="33"/>
-      <c r="I34" s="33"/>
-      <c r="J34" s="33"/>
-      <c r="K34" s="33"/>
-      <c r="L34" s="33"/>
-      <c r="M34" s="33"/>
-      <c r="N34" s="33"/>
-      <c r="O34" s="33"/>
-      <c r="P34" s="33"/>
-      <c r="Q34" s="33"/>
-      <c r="R34" s="33"/>
+      <c r="A34" s="22"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
+      <c r="K34" s="23"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="23"/>
+      <c r="N34" s="23"/>
+      <c r="O34" s="23"/>
+      <c r="P34" s="23"/>
+      <c r="Q34" s="23"/>
+      <c r="R34" s="23"/>
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
       <c r="U34" s="4"/>
@@ -3717,24 +3731,24 @@
       <c r="AT34" s="4"/>
     </row>
     <row r="35" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A35" s="32"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="33"/>
-      <c r="I35" s="33"/>
-      <c r="J35" s="33"/>
-      <c r="K35" s="33"/>
-      <c r="L35" s="33"/>
-      <c r="M35" s="33"/>
-      <c r="N35" s="33"/>
-      <c r="O35" s="33"/>
-      <c r="P35" s="33"/>
-      <c r="Q35" s="33"/>
-      <c r="R35" s="33"/>
+      <c r="A35" s="22"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="23"/>
+      <c r="O35" s="23"/>
+      <c r="P35" s="23"/>
+      <c r="Q35" s="23"/>
+      <c r="R35" s="23"/>
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
       <c r="U35" s="4"/>
@@ -3765,24 +3779,24 @@
       <c r="AT35" s="4"/>
     </row>
     <row r="36" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A36" s="32"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="33"/>
-      <c r="J36" s="33"/>
-      <c r="K36" s="33"/>
-      <c r="L36" s="33"/>
-      <c r="M36" s="33"/>
-      <c r="N36" s="33"/>
-      <c r="O36" s="33"/>
-      <c r="P36" s="33"/>
-      <c r="Q36" s="33"/>
-      <c r="R36" s="33"/>
+      <c r="A36" s="22"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="23"/>
+      <c r="O36" s="23"/>
+      <c r="P36" s="23"/>
+      <c r="Q36" s="23"/>
+      <c r="R36" s="23"/>
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
       <c r="U36" s="4"/>
@@ -3813,24 +3827,24 @@
       <c r="AT36" s="4"/>
     </row>
     <row r="37" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A37" s="32"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
-      <c r="H37" s="33"/>
-      <c r="I37" s="33"/>
-      <c r="J37" s="33"/>
-      <c r="K37" s="33"/>
-      <c r="L37" s="33"/>
-      <c r="M37" s="33"/>
-      <c r="N37" s="33"/>
-      <c r="O37" s="33"/>
-      <c r="P37" s="33"/>
-      <c r="Q37" s="33"/>
-      <c r="R37" s="33"/>
+      <c r="A37" s="22"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="23"/>
+      <c r="N37" s="23"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="23"/>
+      <c r="Q37" s="23"/>
+      <c r="R37" s="23"/>
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
       <c r="U37" s="4"/>
@@ -3861,24 +3875,24 @@
       <c r="AT37" s="4"/>
     </row>
     <row r="38" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A38" s="32"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="33"/>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-      <c r="H38" s="33"/>
-      <c r="I38" s="33"/>
-      <c r="J38" s="33"/>
-      <c r="K38" s="33"/>
-      <c r="L38" s="33"/>
-      <c r="M38" s="33"/>
-      <c r="N38" s="33"/>
-      <c r="O38" s="33"/>
-      <c r="P38" s="33"/>
-      <c r="Q38" s="33"/>
-      <c r="R38" s="33"/>
+      <c r="A38" s="22"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
+      <c r="M38" s="23"/>
+      <c r="N38" s="23"/>
+      <c r="O38" s="23"/>
+      <c r="P38" s="23"/>
+      <c r="Q38" s="23"/>
+      <c r="R38" s="23"/>
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
       <c r="U38" s="4"/>
@@ -3909,24 +3923,24 @@
       <c r="AT38" s="4"/>
     </row>
     <row r="39" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A39" s="32"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="33"/>
-      <c r="I39" s="33"/>
-      <c r="J39" s="33"/>
-      <c r="K39" s="33"/>
-      <c r="L39" s="33"/>
-      <c r="M39" s="33"/>
-      <c r="N39" s="33"/>
-      <c r="O39" s="33"/>
-      <c r="P39" s="33"/>
-      <c r="Q39" s="33"/>
-      <c r="R39" s="33"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="23"/>
+      <c r="K39" s="23"/>
+      <c r="L39" s="23"/>
+      <c r="M39" s="23"/>
+      <c r="N39" s="23"/>
+      <c r="O39" s="23"/>
+      <c r="P39" s="23"/>
+      <c r="Q39" s="23"/>
+      <c r="R39" s="23"/>
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
       <c r="U39" s="4"/>
@@ -3957,24 +3971,24 @@
       <c r="AT39" s="4"/>
     </row>
     <row r="40" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A40" s="32"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="33"/>
-      <c r="H40" s="33"/>
-      <c r="I40" s="33"/>
-      <c r="J40" s="33"/>
-      <c r="K40" s="33"/>
-      <c r="L40" s="33"/>
-      <c r="M40" s="33"/>
-      <c r="N40" s="33"/>
-      <c r="O40" s="33"/>
-      <c r="P40" s="33"/>
-      <c r="Q40" s="33"/>
-      <c r="R40" s="33"/>
+      <c r="A40" s="22"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="23"/>
+      <c r="L40" s="23"/>
+      <c r="M40" s="23"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="23"/>
+      <c r="Q40" s="23"/>
+      <c r="R40" s="23"/>
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
       <c r="U40" s="4"/>
@@ -4005,24 +4019,24 @@
       <c r="AT40" s="4"/>
     </row>
     <row r="41" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A41" s="32"/>
-      <c r="B41" s="33"/>
-      <c r="C41" s="33"/>
-      <c r="D41" s="33"/>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
-      <c r="G41" s="33"/>
-      <c r="H41" s="33"/>
-      <c r="I41" s="33"/>
-      <c r="J41" s="33"/>
-      <c r="K41" s="33"/>
-      <c r="L41" s="33"/>
-      <c r="M41" s="33"/>
-      <c r="N41" s="33"/>
-      <c r="O41" s="33"/>
-      <c r="P41" s="33"/>
-      <c r="Q41" s="33"/>
-      <c r="R41" s="33"/>
+      <c r="A41" s="22"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="23"/>
+      <c r="Q41" s="23"/>
+      <c r="R41" s="23"/>
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
       <c r="U41" s="4"/>
@@ -4053,24 +4067,24 @@
       <c r="AT41" s="4"/>
     </row>
     <row r="42" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A42" s="32"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="33"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="33"/>
-      <c r="I42" s="33"/>
-      <c r="J42" s="33"/>
-      <c r="K42" s="33"/>
-      <c r="L42" s="33"/>
-      <c r="M42" s="33"/>
-      <c r="N42" s="33"/>
-      <c r="O42" s="33"/>
-      <c r="P42" s="33"/>
-      <c r="Q42" s="33"/>
-      <c r="R42" s="33"/>
+      <c r="A42" s="22"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+      <c r="P42" s="23"/>
+      <c r="Q42" s="23"/>
+      <c r="R42" s="23"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
       <c r="U42" s="4"/>
@@ -4101,24 +4115,24 @@
       <c r="AT42" s="4"/>
     </row>
     <row r="43" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A43" s="32"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="33"/>
-      <c r="H43" s="33"/>
-      <c r="I43" s="33"/>
-      <c r="J43" s="33"/>
-      <c r="K43" s="33"/>
-      <c r="L43" s="33"/>
-      <c r="M43" s="33"/>
-      <c r="N43" s="33"/>
-      <c r="O43" s="33"/>
-      <c r="P43" s="33"/>
-      <c r="Q43" s="33"/>
-      <c r="R43" s="33"/>
+      <c r="A43" s="22"/>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="23"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="23"/>
+      <c r="K43" s="23"/>
+      <c r="L43" s="23"/>
+      <c r="M43" s="23"/>
+      <c r="N43" s="23"/>
+      <c r="O43" s="23"/>
+      <c r="P43" s="23"/>
+      <c r="Q43" s="23"/>
+      <c r="R43" s="23"/>
       <c r="S43" s="4"/>
       <c r="T43" s="4"/>
       <c r="U43" s="4"/>
@@ -4149,24 +4163,24 @@
       <c r="AT43" s="4"/>
     </row>
     <row r="44" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A44" s="32"/>
-      <c r="B44" s="33"/>
-      <c r="C44" s="33"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="33"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="33"/>
-      <c r="I44" s="33"/>
-      <c r="J44" s="33"/>
-      <c r="K44" s="33"/>
-      <c r="L44" s="33"/>
-      <c r="M44" s="33"/>
-      <c r="N44" s="33"/>
-      <c r="O44" s="33"/>
-      <c r="P44" s="33"/>
-      <c r="Q44" s="33"/>
-      <c r="R44" s="33"/>
+      <c r="A44" s="22"/>
+      <c r="B44" s="23"/>
+      <c r="C44" s="23"/>
+      <c r="D44" s="23"/>
+      <c r="E44" s="23"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="23"/>
+      <c r="K44" s="23"/>
+      <c r="L44" s="23"/>
+      <c r="M44" s="23"/>
+      <c r="N44" s="23"/>
+      <c r="O44" s="23"/>
+      <c r="P44" s="23"/>
+      <c r="Q44" s="23"/>
+      <c r="R44" s="23"/>
       <c r="S44" s="4"/>
       <c r="T44" s="4"/>
       <c r="U44" s="4"/>
@@ -4197,24 +4211,24 @@
       <c r="AT44" s="4"/>
     </row>
     <row r="45" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A45" s="32"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="33"/>
-      <c r="D45" s="33"/>
-      <c r="E45" s="33"/>
-      <c r="F45" s="33"/>
-      <c r="G45" s="33"/>
-      <c r="H45" s="33"/>
-      <c r="I45" s="33"/>
-      <c r="J45" s="33"/>
-      <c r="K45" s="33"/>
-      <c r="L45" s="33"/>
-      <c r="M45" s="33"/>
-      <c r="N45" s="33"/>
-      <c r="O45" s="33"/>
-      <c r="P45" s="33"/>
-      <c r="Q45" s="33"/>
-      <c r="R45" s="33"/>
+      <c r="A45" s="22"/>
+      <c r="B45" s="23"/>
+      <c r="C45" s="23"/>
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="23"/>
+      <c r="K45" s="23"/>
+      <c r="L45" s="23"/>
+      <c r="M45" s="23"/>
+      <c r="N45" s="23"/>
+      <c r="O45" s="23"/>
+      <c r="P45" s="23"/>
+      <c r="Q45" s="23"/>
+      <c r="R45" s="23"/>
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
       <c r="U45" s="4"/>
@@ -4245,24 +4259,24 @@
       <c r="AT45" s="4"/>
     </row>
     <row r="46" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A46" s="32"/>
-      <c r="B46" s="33"/>
-      <c r="C46" s="33"/>
-      <c r="D46" s="33"/>
-      <c r="E46" s="33"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="33"/>
-      <c r="H46" s="33"/>
-      <c r="I46" s="33"/>
-      <c r="J46" s="33"/>
-      <c r="K46" s="33"/>
-      <c r="L46" s="33"/>
-      <c r="M46" s="33"/>
-      <c r="N46" s="33"/>
-      <c r="O46" s="33"/>
-      <c r="P46" s="33"/>
-      <c r="Q46" s="33"/>
-      <c r="R46" s="33"/>
+      <c r="A46" s="22"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
+      <c r="M46" s="23"/>
+      <c r="N46" s="23"/>
+      <c r="O46" s="23"/>
+      <c r="P46" s="23"/>
+      <c r="Q46" s="23"/>
+      <c r="R46" s="23"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
       <c r="U46" s="4"/>
@@ -4293,24 +4307,24 @@
       <c r="AT46" s="4"/>
     </row>
     <row r="47" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A47" s="32"/>
-      <c r="B47" s="33"/>
-      <c r="C47" s="33"/>
-      <c r="D47" s="33"/>
-      <c r="E47" s="33"/>
-      <c r="F47" s="33"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="33"/>
-      <c r="I47" s="33"/>
-      <c r="J47" s="33"/>
-      <c r="K47" s="33"/>
-      <c r="L47" s="33"/>
-      <c r="M47" s="33"/>
-      <c r="N47" s="33"/>
-      <c r="O47" s="33"/>
-      <c r="P47" s="33"/>
-      <c r="Q47" s="33"/>
-      <c r="R47" s="33"/>
+      <c r="A47" s="22"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23"/>
+      <c r="K47" s="23"/>
+      <c r="L47" s="23"/>
+      <c r="M47" s="23"/>
+      <c r="N47" s="23"/>
+      <c r="O47" s="23"/>
+      <c r="P47" s="23"/>
+      <c r="Q47" s="23"/>
+      <c r="R47" s="23"/>
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
       <c r="U47" s="4"/>
@@ -4341,24 +4355,24 @@
       <c r="AT47" s="4"/>
     </row>
     <row r="48" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A48" s="32"/>
-      <c r="B48" s="33"/>
-      <c r="C48" s="33"/>
-      <c r="D48" s="33"/>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="33"/>
-      <c r="J48" s="33"/>
-      <c r="K48" s="33"/>
-      <c r="L48" s="33"/>
-      <c r="M48" s="33"/>
-      <c r="N48" s="33"/>
-      <c r="O48" s="33"/>
-      <c r="P48" s="33"/>
-      <c r="Q48" s="33"/>
-      <c r="R48" s="33"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
+      <c r="H48" s="23"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="23"/>
+      <c r="K48" s="23"/>
+      <c r="L48" s="23"/>
+      <c r="M48" s="23"/>
+      <c r="N48" s="23"/>
+      <c r="O48" s="23"/>
+      <c r="P48" s="23"/>
+      <c r="Q48" s="23"/>
+      <c r="R48" s="23"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
       <c r="U48" s="4"/>
@@ -4389,24 +4403,24 @@
       <c r="AT48" s="4"/>
     </row>
     <row r="49" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A49" s="32"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="33"/>
-      <c r="D49" s="33"/>
-      <c r="E49" s="33"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="33"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="33"/>
-      <c r="J49" s="33"/>
-      <c r="K49" s="33"/>
-      <c r="L49" s="33"/>
-      <c r="M49" s="33"/>
-      <c r="N49" s="33"/>
-      <c r="O49" s="33"/>
-      <c r="P49" s="33"/>
-      <c r="Q49" s="33"/>
-      <c r="R49" s="33"/>
+      <c r="A49" s="22"/>
+      <c r="B49" s="23"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="23"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="23"/>
+      <c r="H49" s="23"/>
+      <c r="I49" s="23"/>
+      <c r="J49" s="23"/>
+      <c r="K49" s="23"/>
+      <c r="L49" s="23"/>
+      <c r="M49" s="23"/>
+      <c r="N49" s="23"/>
+      <c r="O49" s="23"/>
+      <c r="P49" s="23"/>
+      <c r="Q49" s="23"/>
+      <c r="R49" s="23"/>
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
       <c r="U49" s="4"/>
@@ -4437,24 +4451,24 @@
       <c r="AT49" s="4"/>
     </row>
     <row r="50" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A50" s="32"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="33"/>
-      <c r="D50" s="33"/>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="33"/>
-      <c r="H50" s="33"/>
-      <c r="I50" s="33"/>
-      <c r="J50" s="33"/>
-      <c r="K50" s="33"/>
-      <c r="L50" s="33"/>
-      <c r="M50" s="33"/>
-      <c r="N50" s="33"/>
-      <c r="O50" s="33"/>
-      <c r="P50" s="33"/>
-      <c r="Q50" s="33"/>
-      <c r="R50" s="33"/>
+      <c r="A50" s="22"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="23"/>
+      <c r="H50" s="23"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="23"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
+      <c r="M50" s="23"/>
+      <c r="N50" s="23"/>
+      <c r="O50" s="23"/>
+      <c r="P50" s="23"/>
+      <c r="Q50" s="23"/>
+      <c r="R50" s="23"/>
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
       <c r="U50" s="4"/>
@@ -4485,24 +4499,24 @@
       <c r="AT50" s="4"/>
     </row>
     <row r="51" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A51" s="32"/>
-      <c r="B51" s="33"/>
-      <c r="C51" s="33"/>
-      <c r="D51" s="33"/>
-      <c r="E51" s="33"/>
-      <c r="F51" s="33"/>
-      <c r="G51" s="33"/>
-      <c r="H51" s="33"/>
-      <c r="I51" s="33"/>
-      <c r="J51" s="33"/>
-      <c r="K51" s="33"/>
-      <c r="L51" s="33"/>
-      <c r="M51" s="33"/>
-      <c r="N51" s="33"/>
-      <c r="O51" s="33"/>
-      <c r="P51" s="33"/>
-      <c r="Q51" s="33"/>
-      <c r="R51" s="33"/>
+      <c r="A51" s="22"/>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="23"/>
+      <c r="H51" s="23"/>
+      <c r="I51" s="23"/>
+      <c r="J51" s="23"/>
+      <c r="K51" s="23"/>
+      <c r="L51" s="23"/>
+      <c r="M51" s="23"/>
+      <c r="N51" s="23"/>
+      <c r="O51" s="23"/>
+      <c r="P51" s="23"/>
+      <c r="Q51" s="23"/>
+      <c r="R51" s="23"/>
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
       <c r="U51" s="4"/>
@@ -4533,24 +4547,24 @@
       <c r="AT51" s="4"/>
     </row>
     <row r="52" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A52" s="32"/>
-      <c r="B52" s="33"/>
-      <c r="C52" s="33"/>
-      <c r="D52" s="33"/>
-      <c r="E52" s="33"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="33"/>
-      <c r="H52" s="33"/>
-      <c r="I52" s="33"/>
-      <c r="J52" s="33"/>
-      <c r="K52" s="33"/>
-      <c r="L52" s="33"/>
-      <c r="M52" s="33"/>
-      <c r="N52" s="33"/>
-      <c r="O52" s="33"/>
-      <c r="P52" s="33"/>
-      <c r="Q52" s="33"/>
-      <c r="R52" s="33"/>
+      <c r="A52" s="22"/>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="23"/>
+      <c r="I52" s="23"/>
+      <c r="J52" s="23"/>
+      <c r="K52" s="23"/>
+      <c r="L52" s="23"/>
+      <c r="M52" s="23"/>
+      <c r="N52" s="23"/>
+      <c r="O52" s="23"/>
+      <c r="P52" s="23"/>
+      <c r="Q52" s="23"/>
+      <c r="R52" s="23"/>
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
       <c r="U52" s="4"/>
@@ -4581,24 +4595,24 @@
       <c r="AT52" s="4"/>
     </row>
     <row r="53" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A53" s="32"/>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33"/>
-      <c r="D53" s="33"/>
-      <c r="E53" s="33"/>
-      <c r="F53" s="33"/>
-      <c r="G53" s="33"/>
-      <c r="H53" s="33"/>
-      <c r="I53" s="33"/>
-      <c r="J53" s="33"/>
-      <c r="K53" s="33"/>
-      <c r="L53" s="33"/>
-      <c r="M53" s="33"/>
-      <c r="N53" s="33"/>
-      <c r="O53" s="33"/>
-      <c r="P53" s="33"/>
-      <c r="Q53" s="33"/>
-      <c r="R53" s="33"/>
+      <c r="A53" s="22"/>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="23"/>
+      <c r="I53" s="23"/>
+      <c r="J53" s="23"/>
+      <c r="K53" s="23"/>
+      <c r="L53" s="23"/>
+      <c r="M53" s="23"/>
+      <c r="N53" s="23"/>
+      <c r="O53" s="23"/>
+      <c r="P53" s="23"/>
+      <c r="Q53" s="23"/>
+      <c r="R53" s="23"/>
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
       <c r="U53" s="4"/>
@@ -4629,24 +4643,24 @@
       <c r="AT53" s="4"/>
     </row>
     <row r="54" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A54" s="32"/>
-      <c r="B54" s="33"/>
-      <c r="C54" s="33"/>
-      <c r="D54" s="33"/>
-      <c r="E54" s="33"/>
-      <c r="F54" s="33"/>
-      <c r="G54" s="33"/>
-      <c r="H54" s="33"/>
-      <c r="I54" s="33"/>
-      <c r="J54" s="33"/>
-      <c r="K54" s="33"/>
-      <c r="L54" s="33"/>
-      <c r="M54" s="33"/>
-      <c r="N54" s="33"/>
-      <c r="O54" s="33"/>
-      <c r="P54" s="33"/>
-      <c r="Q54" s="33"/>
-      <c r="R54" s="33"/>
+      <c r="A54" s="22"/>
+      <c r="B54" s="23"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="23"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="23"/>
+      <c r="I54" s="23"/>
+      <c r="J54" s="23"/>
+      <c r="K54" s="23"/>
+      <c r="L54" s="23"/>
+      <c r="M54" s="23"/>
+      <c r="N54" s="23"/>
+      <c r="O54" s="23"/>
+      <c r="P54" s="23"/>
+      <c r="Q54" s="23"/>
+      <c r="R54" s="23"/>
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
       <c r="U54" s="4"/>
@@ -4677,24 +4691,24 @@
       <c r="AT54" s="4"/>
     </row>
     <row r="55" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A55" s="32"/>
-      <c r="B55" s="33"/>
-      <c r="C55" s="33"/>
-      <c r="D55" s="33"/>
-      <c r="E55" s="33"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="33"/>
-      <c r="H55" s="33"/>
-      <c r="I55" s="33"/>
-      <c r="J55" s="33"/>
-      <c r="K55" s="33"/>
-      <c r="L55" s="33"/>
-      <c r="M55" s="33"/>
-      <c r="N55" s="33"/>
-      <c r="O55" s="33"/>
-      <c r="P55" s="33"/>
-      <c r="Q55" s="33"/>
-      <c r="R55" s="33"/>
+      <c r="A55" s="22"/>
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
+      <c r="H55" s="23"/>
+      <c r="I55" s="23"/>
+      <c r="J55" s="23"/>
+      <c r="K55" s="23"/>
+      <c r="L55" s="23"/>
+      <c r="M55" s="23"/>
+      <c r="N55" s="23"/>
+      <c r="O55" s="23"/>
+      <c r="P55" s="23"/>
+      <c r="Q55" s="23"/>
+      <c r="R55" s="23"/>
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
       <c r="U55" s="4"/>
@@ -4725,24 +4739,24 @@
       <c r="AT55" s="4"/>
     </row>
     <row r="56" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A56" s="32"/>
-      <c r="B56" s="33"/>
-      <c r="C56" s="33"/>
-      <c r="D56" s="33"/>
-      <c r="E56" s="33"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="33"/>
-      <c r="H56" s="33"/>
-      <c r="I56" s="33"/>
-      <c r="J56" s="33"/>
-      <c r="K56" s="33"/>
-      <c r="L56" s="33"/>
-      <c r="M56" s="33"/>
-      <c r="N56" s="33"/>
-      <c r="O56" s="33"/>
-      <c r="P56" s="33"/>
-      <c r="Q56" s="33"/>
-      <c r="R56" s="33"/>
+      <c r="A56" s="22"/>
+      <c r="B56" s="23"/>
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="23"/>
+      <c r="H56" s="23"/>
+      <c r="I56" s="23"/>
+      <c r="J56" s="23"/>
+      <c r="K56" s="23"/>
+      <c r="L56" s="23"/>
+      <c r="M56" s="23"/>
+      <c r="N56" s="23"/>
+      <c r="O56" s="23"/>
+      <c r="P56" s="23"/>
+      <c r="Q56" s="23"/>
+      <c r="R56" s="23"/>
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
       <c r="U56" s="4"/>
@@ -4773,24 +4787,24 @@
       <c r="AT56" s="4"/>
     </row>
     <row r="57" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A57" s="32"/>
-      <c r="B57" s="33"/>
-      <c r="C57" s="33"/>
-      <c r="D57" s="33"/>
-      <c r="E57" s="33"/>
-      <c r="F57" s="33"/>
-      <c r="G57" s="33"/>
-      <c r="H57" s="33"/>
-      <c r="I57" s="33"/>
-      <c r="J57" s="33"/>
-      <c r="K57" s="33"/>
-      <c r="L57" s="33"/>
-      <c r="M57" s="33"/>
-      <c r="N57" s="33"/>
-      <c r="O57" s="33"/>
-      <c r="P57" s="33"/>
-      <c r="Q57" s="33"/>
-      <c r="R57" s="33"/>
+      <c r="A57" s="22"/>
+      <c r="B57" s="23"/>
+      <c r="C57" s="23"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="23"/>
+      <c r="F57" s="23"/>
+      <c r="G57" s="23"/>
+      <c r="H57" s="23"/>
+      <c r="I57" s="23"/>
+      <c r="J57" s="23"/>
+      <c r="K57" s="23"/>
+      <c r="L57" s="23"/>
+      <c r="M57" s="23"/>
+      <c r="N57" s="23"/>
+      <c r="O57" s="23"/>
+      <c r="P57" s="23"/>
+      <c r="Q57" s="23"/>
+      <c r="R57" s="23"/>
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
       <c r="U57" s="4"/>
@@ -4821,24 +4835,24 @@
       <c r="AT57" s="4"/>
     </row>
     <row r="58" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A58" s="32"/>
-      <c r="B58" s="33"/>
-      <c r="C58" s="33"/>
-      <c r="D58" s="33"/>
-      <c r="E58" s="33"/>
-      <c r="F58" s="33"/>
-      <c r="G58" s="33"/>
-      <c r="H58" s="33"/>
-      <c r="I58" s="33"/>
-      <c r="J58" s="33"/>
-      <c r="K58" s="33"/>
-      <c r="L58" s="33"/>
-      <c r="M58" s="33"/>
-      <c r="N58" s="33"/>
-      <c r="O58" s="33"/>
-      <c r="P58" s="33"/>
-      <c r="Q58" s="33"/>
-      <c r="R58" s="33"/>
+      <c r="A58" s="22"/>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="23"/>
+      <c r="F58" s="23"/>
+      <c r="G58" s="23"/>
+      <c r="H58" s="23"/>
+      <c r="I58" s="23"/>
+      <c r="J58" s="23"/>
+      <c r="K58" s="23"/>
+      <c r="L58" s="23"/>
+      <c r="M58" s="23"/>
+      <c r="N58" s="23"/>
+      <c r="O58" s="23"/>
+      <c r="P58" s="23"/>
+      <c r="Q58" s="23"/>
+      <c r="R58" s="23"/>
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
       <c r="U58" s="4"/>
@@ -4869,24 +4883,24 @@
       <c r="AT58" s="4"/>
     </row>
     <row r="59" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A59" s="32"/>
-      <c r="B59" s="33"/>
-      <c r="C59" s="33"/>
-      <c r="D59" s="33"/>
-      <c r="E59" s="33"/>
-      <c r="F59" s="33"/>
-      <c r="G59" s="33"/>
-      <c r="H59" s="33"/>
-      <c r="I59" s="33"/>
-      <c r="J59" s="33"/>
-      <c r="K59" s="33"/>
-      <c r="L59" s="33"/>
-      <c r="M59" s="33"/>
-      <c r="N59" s="33"/>
-      <c r="O59" s="33"/>
-      <c r="P59" s="33"/>
-      <c r="Q59" s="33"/>
-      <c r="R59" s="33"/>
+      <c r="A59" s="22"/>
+      <c r="B59" s="23"/>
+      <c r="C59" s="23"/>
+      <c r="D59" s="23"/>
+      <c r="E59" s="23"/>
+      <c r="F59" s="23"/>
+      <c r="G59" s="23"/>
+      <c r="H59" s="23"/>
+      <c r="I59" s="23"/>
+      <c r="J59" s="23"/>
+      <c r="K59" s="23"/>
+      <c r="L59" s="23"/>
+      <c r="M59" s="23"/>
+      <c r="N59" s="23"/>
+      <c r="O59" s="23"/>
+      <c r="P59" s="23"/>
+      <c r="Q59" s="23"/>
+      <c r="R59" s="23"/>
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
       <c r="U59" s="4"/>
@@ -4917,24 +4931,24 @@
       <c r="AT59" s="4"/>
     </row>
     <row r="60" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A60" s="32"/>
-      <c r="B60" s="33"/>
-      <c r="C60" s="33"/>
-      <c r="D60" s="33"/>
-      <c r="E60" s="33"/>
-      <c r="F60" s="33"/>
-      <c r="G60" s="33"/>
-      <c r="H60" s="33"/>
-      <c r="I60" s="33"/>
-      <c r="J60" s="33"/>
-      <c r="K60" s="33"/>
-      <c r="L60" s="33"/>
-      <c r="M60" s="33"/>
-      <c r="N60" s="33"/>
-      <c r="O60" s="33"/>
-      <c r="P60" s="33"/>
-      <c r="Q60" s="33"/>
-      <c r="R60" s="33"/>
+      <c r="A60" s="22"/>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="23"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="23"/>
+      <c r="H60" s="23"/>
+      <c r="I60" s="23"/>
+      <c r="J60" s="23"/>
+      <c r="K60" s="23"/>
+      <c r="L60" s="23"/>
+      <c r="M60" s="23"/>
+      <c r="N60" s="23"/>
+      <c r="O60" s="23"/>
+      <c r="P60" s="23"/>
+      <c r="Q60" s="23"/>
+      <c r="R60" s="23"/>
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
       <c r="U60" s="4"/>
@@ -4965,44 +4979,44 @@
       <c r="AT60" s="4"/>
     </row>
     <row r="61" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A61" s="32"/>
-      <c r="B61" s="33"/>
-      <c r="C61" s="33"/>
-      <c r="D61" s="33"/>
-      <c r="E61" s="33"/>
-      <c r="F61" s="33"/>
-      <c r="G61" s="33"/>
-      <c r="H61" s="33"/>
-      <c r="I61" s="33"/>
-      <c r="J61" s="33"/>
-      <c r="K61" s="33"/>
-      <c r="L61" s="33"/>
-      <c r="M61" s="33"/>
-      <c r="N61" s="33"/>
-      <c r="O61" s="33"/>
-      <c r="P61" s="33"/>
-      <c r="Q61" s="33"/>
-      <c r="R61" s="33"/>
+      <c r="A61" s="22"/>
+      <c r="B61" s="23"/>
+      <c r="C61" s="23"/>
+      <c r="D61" s="23"/>
+      <c r="E61" s="23"/>
+      <c r="F61" s="23"/>
+      <c r="G61" s="23"/>
+      <c r="H61" s="23"/>
+      <c r="I61" s="23"/>
+      <c r="J61" s="23"/>
+      <c r="K61" s="23"/>
+      <c r="L61" s="23"/>
+      <c r="M61" s="23"/>
+      <c r="N61" s="23"/>
+      <c r="O61" s="23"/>
+      <c r="P61" s="23"/>
+      <c r="Q61" s="23"/>
+      <c r="R61" s="23"/>
     </row>
     <row r="62" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A62" s="32"/>
-      <c r="B62" s="33"/>
-      <c r="C62" s="33"/>
-      <c r="D62" s="33"/>
-      <c r="E62" s="33"/>
-      <c r="F62" s="33"/>
-      <c r="G62" s="33"/>
-      <c r="H62" s="33"/>
-      <c r="I62" s="33"/>
-      <c r="J62" s="33"/>
-      <c r="K62" s="33"/>
-      <c r="L62" s="33"/>
-      <c r="M62" s="33"/>
-      <c r="N62" s="33"/>
-      <c r="O62" s="33"/>
-      <c r="P62" s="33"/>
-      <c r="Q62" s="33"/>
-      <c r="R62" s="33"/>
+      <c r="A62" s="22"/>
+      <c r="B62" s="23"/>
+      <c r="C62" s="23"/>
+      <c r="D62" s="23"/>
+      <c r="E62" s="23"/>
+      <c r="F62" s="23"/>
+      <c r="G62" s="23"/>
+      <c r="H62" s="23"/>
+      <c r="I62" s="23"/>
+      <c r="J62" s="23"/>
+      <c r="K62" s="23"/>
+      <c r="L62" s="23"/>
+      <c r="M62" s="23"/>
+      <c r="N62" s="23"/>
+      <c r="O62" s="23"/>
+      <c r="P62" s="23"/>
+      <c r="Q62" s="23"/>
+      <c r="R62" s="23"/>
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
       <c r="U62" s="4"/>
@@ -5033,24 +5047,24 @@
       <c r="AT62" s="4"/>
     </row>
     <row r="63" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A63" s="32"/>
-      <c r="B63" s="33"/>
-      <c r="C63" s="33"/>
-      <c r="D63" s="33"/>
-      <c r="E63" s="33"/>
-      <c r="F63" s="33"/>
-      <c r="G63" s="33"/>
-      <c r="H63" s="33"/>
-      <c r="I63" s="33"/>
-      <c r="J63" s="33"/>
-      <c r="K63" s="33"/>
-      <c r="L63" s="33"/>
-      <c r="M63" s="33"/>
-      <c r="N63" s="33"/>
-      <c r="O63" s="33"/>
-      <c r="P63" s="33"/>
-      <c r="Q63" s="33"/>
-      <c r="R63" s="33"/>
+      <c r="A63" s="22"/>
+      <c r="B63" s="23"/>
+      <c r="C63" s="23"/>
+      <c r="D63" s="23"/>
+      <c r="E63" s="23"/>
+      <c r="F63" s="23"/>
+      <c r="G63" s="23"/>
+      <c r="H63" s="23"/>
+      <c r="I63" s="23"/>
+      <c r="J63" s="23"/>
+      <c r="K63" s="23"/>
+      <c r="L63" s="23"/>
+      <c r="M63" s="23"/>
+      <c r="N63" s="23"/>
+      <c r="O63" s="23"/>
+      <c r="P63" s="23"/>
+      <c r="Q63" s="23"/>
+      <c r="R63" s="23"/>
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
       <c r="U63" s="4"/>
@@ -5081,24 +5095,24 @@
       <c r="AT63" s="4"/>
     </row>
     <row r="64" spans="1:46" ht="80.099999999999994" customHeight="1">
-      <c r="A64" s="32"/>
-      <c r="B64" s="33"/>
-      <c r="C64" s="33"/>
-      <c r="D64" s="33"/>
-      <c r="E64" s="33"/>
-      <c r="F64" s="33"/>
-      <c r="G64" s="33"/>
-      <c r="H64" s="33"/>
-      <c r="I64" s="33"/>
-      <c r="J64" s="33"/>
-      <c r="K64" s="33"/>
-      <c r="L64" s="33"/>
-      <c r="M64" s="33"/>
-      <c r="N64" s="33"/>
-      <c r="O64" s="33"/>
-      <c r="P64" s="33"/>
-      <c r="Q64" s="33"/>
-      <c r="R64" s="33"/>
+      <c r="A64" s="22"/>
+      <c r="B64" s="23"/>
+      <c r="C64" s="23"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="23"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="23"/>
+      <c r="I64" s="23"/>
+      <c r="J64" s="23"/>
+      <c r="K64" s="23"/>
+      <c r="L64" s="23"/>
+      <c r="M64" s="23"/>
+      <c r="N64" s="23"/>
+      <c r="O64" s="23"/>
+      <c r="P64" s="23"/>
+      <c r="Q64" s="23"/>
+      <c r="R64" s="23"/>
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
       <c r="U64" s="4"/>
@@ -8037,13 +8051,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A21:R64"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A3:A4"/>
@@ -8053,6 +8060,13 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="J3:J4"/>
+    <mergeCell ref="A21:R64"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="10" orientation="portrait" r:id="rId1"/>

</xml_diff>